<commit_message>
add cal and alternate imig_prev
</commit_message>
<xml_diff>
--- a/calibrations/Y-factors/hbv_hepaus_calibrations.xlsx
+++ b/calibrations/Y-factors/hbv_hepaus_calibrations.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="184">
   <si>
     <t>meta_y_factor</t>
   </si>
@@ -133,171 +133,180 @@
     <t>acm</t>
   </si>
   <si>
+    <t>mig_rate</t>
+  </si>
+  <si>
+    <t>hepb_prev</t>
+  </si>
+  <si>
+    <t>diagnosed_meas</t>
+  </si>
+  <si>
+    <t>linked_meas</t>
+  </si>
+  <si>
+    <t>treat_cov</t>
+  </si>
+  <si>
+    <t>epos_total</t>
+  </si>
+  <si>
+    <t>hep_dth</t>
+  </si>
+  <si>
+    <t>imig_vax_prop</t>
+  </si>
+  <si>
+    <t>imig_clr_prop</t>
+  </si>
+  <si>
+    <t>tx_chb_cc</t>
+  </si>
+  <si>
+    <t>tx_chb_hcc</t>
+  </si>
+  <si>
+    <t>tx_cir_hcc</t>
+  </si>
+  <si>
+    <t>tx_cc_dc</t>
+  </si>
+  <si>
+    <t>dc_cc_t</t>
+  </si>
+  <si>
+    <t>tx_dc_death</t>
+  </si>
+  <si>
+    <t>sh_si_t</t>
+  </si>
+  <si>
+    <t>eh_si</t>
+  </si>
+  <si>
+    <t>acu_chb</t>
+  </si>
+  <si>
+    <t>acu_dth</t>
+  </si>
+  <si>
+    <t>ei_eh</t>
+  </si>
+  <si>
+    <t>si_sh</t>
+  </si>
+  <si>
+    <t>sh_si</t>
+  </si>
+  <si>
+    <t>eh_cc_in</t>
+  </si>
+  <si>
+    <t>sh_cc_in</t>
+  </si>
+  <si>
+    <t>cc_dc</t>
+  </si>
+  <si>
+    <t>ei_hcc_in</t>
+  </si>
+  <si>
+    <t>act_hcc_in</t>
+  </si>
+  <si>
+    <t>si_hcc_in</t>
+  </si>
+  <si>
+    <t>cir_hcc_in</t>
+  </si>
+  <si>
+    <t>dc_dth</t>
+  </si>
+  <si>
+    <t>hcc_dth</t>
+  </si>
+  <si>
+    <t>chb_clr</t>
+  </si>
+  <si>
+    <t>y_hcc</t>
+  </si>
+  <si>
+    <t>y_cc</t>
+  </si>
+  <si>
+    <t>foi_cal</t>
+  </si>
+  <si>
+    <t>anc_scr</t>
+  </si>
+  <si>
+    <t>pregs</t>
+  </si>
+  <si>
+    <t>nullipar</t>
+  </si>
+  <si>
+    <t>preg_ltc_rate</t>
+  </si>
+  <si>
+    <t>ve_hepbd_lvl</t>
+  </si>
+  <si>
+    <t>ve_hepbd_hvl</t>
+  </si>
+  <si>
+    <t>ve_hepbd_pap</t>
+  </si>
+  <si>
+    <t>ve_hepb3</t>
+  </si>
+  <si>
+    <t>mtct_chb</t>
+  </si>
+  <si>
+    <t>trisk_low</t>
+  </si>
+  <si>
+    <t>trisk_high</t>
+  </si>
+  <si>
+    <t>hepbd_cov</t>
+  </si>
+  <si>
+    <t>hepb3_cov</t>
+  </si>
+  <si>
+    <t>hvl_epos</t>
+  </si>
+  <si>
+    <t>hvl_eneg</t>
+  </si>
+  <si>
+    <t>ts_rate</t>
+  </si>
+  <si>
+    <t>ltf_rate</t>
+  </si>
+  <si>
+    <t>diag_measure</t>
+  </si>
+  <si>
+    <t>ltc_measure</t>
+  </si>
+  <si>
+    <t>treat_measure</t>
+  </si>
+  <si>
+    <t>imig_rate</t>
+  </si>
+  <si>
     <t>emig_rate</t>
   </si>
   <si>
-    <t>hepb_prev</t>
-  </si>
-  <si>
-    <t>diagnosed_meas</t>
-  </si>
-  <si>
-    <t>linked_meas</t>
-  </si>
-  <si>
-    <t>treat_cov</t>
-  </si>
-  <si>
-    <t>epos_total</t>
-  </si>
-  <si>
-    <t>imig_rate</t>
-  </si>
-  <si>
     <t>imig_prev</t>
   </si>
   <si>
-    <t>imig_vax_prop</t>
-  </si>
-  <si>
-    <t>imig_clr_prop</t>
-  </si>
-  <si>
-    <t>tx_chb_cc</t>
-  </si>
-  <si>
-    <t>tx_chb_hcc</t>
-  </si>
-  <si>
-    <t>tx_cir_hcc</t>
-  </si>
-  <si>
-    <t>tx_cc_dc</t>
-  </si>
-  <si>
-    <t>dc_cc_t</t>
-  </si>
-  <si>
-    <t>tx_dc_death</t>
-  </si>
-  <si>
-    <t>sh_si_t</t>
-  </si>
-  <si>
-    <t>eh_si</t>
-  </si>
-  <si>
-    <t>acu_chb</t>
-  </si>
-  <si>
-    <t>acu_dth</t>
-  </si>
-  <si>
-    <t>ei_eh</t>
-  </si>
-  <si>
-    <t>si_sh</t>
-  </si>
-  <si>
-    <t>sh_si</t>
-  </si>
-  <si>
-    <t>eh_cc_in</t>
-  </si>
-  <si>
-    <t>sh_cc_in</t>
-  </si>
-  <si>
-    <t>cc_dc</t>
-  </si>
-  <si>
-    <t>ei_hcc_in</t>
-  </si>
-  <si>
-    <t>act_hcc_in</t>
-  </si>
-  <si>
-    <t>si_hcc_in</t>
-  </si>
-  <si>
-    <t>cir_hcc_in</t>
-  </si>
-  <si>
-    <t>dc_dth</t>
-  </si>
-  <si>
-    <t>hcc_dth</t>
-  </si>
-  <si>
-    <t>y_hcc</t>
-  </si>
-  <si>
-    <t>y_cc</t>
-  </si>
-  <si>
-    <t>foi_cal</t>
-  </si>
-  <si>
-    <t>anc_scr</t>
-  </si>
-  <si>
-    <t>pregs</t>
-  </si>
-  <si>
-    <t>nullipar</t>
-  </si>
-  <si>
-    <t>preg_ltc_rate</t>
-  </si>
-  <si>
-    <t>ve_hepbd_lvl</t>
-  </si>
-  <si>
-    <t>ve_hepbd_hvl</t>
-  </si>
-  <si>
-    <t>ve_hepbd_pap</t>
-  </si>
-  <si>
-    <t>ve_hepb3</t>
-  </si>
-  <si>
-    <t>mtct_chb</t>
-  </si>
-  <si>
-    <t>trisk_low</t>
-  </si>
-  <si>
-    <t>trisk_high</t>
-  </si>
-  <si>
-    <t>hepbd_cov</t>
-  </si>
-  <si>
-    <t>hepb3_cov</t>
-  </si>
-  <si>
-    <t>hvl_epos</t>
-  </si>
-  <si>
-    <t>hvl_eneg</t>
-  </si>
-  <si>
-    <t>ts_rate</t>
-  </si>
-  <si>
-    <t>ltf_rate</t>
-  </si>
-  <si>
-    <t>diag_measure</t>
-  </si>
-  <si>
-    <t>ltc_measure</t>
-  </si>
-  <si>
-    <t>treat_measure</t>
-  </si>
-  <si>
     <t>imig_rem</t>
   </si>
   <si>
@@ -545,6 +554,9 @@
   </si>
   <si>
     <t>treat_rate</t>
+  </si>
+  <si>
+    <t>inc_hcc</t>
   </si>
   <si>
     <t>mx_mtct</t>
@@ -911,7 +923,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA195"/>
+  <dimension ref="A1:AA200"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:27">
@@ -1897,76 +1909,76 @@
         <v>1</v>
       </c>
       <c r="D13">
+        <v>0.1874999999999999</v>
+      </c>
+      <c r="E13">
         <v>0.9</v>
       </c>
-      <c r="E13">
-        <v>0.975</v>
-      </c>
       <c r="F13">
-        <v>3.053125</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>0.1874999999999999</v>
+        <v>0.1775390625</v>
       </c>
       <c r="H13">
-        <v>0.1</v>
+        <v>0.5499999999999999</v>
       </c>
       <c r="I13">
-        <v>3.1671142578125</v>
+        <v>1</v>
       </c>
       <c r="J13">
+        <v>0.6937500000000001</v>
+      </c>
+      <c r="K13">
+        <v>0.1242187499999999</v>
+      </c>
+      <c r="L13">
+        <v>1.1125</v>
+      </c>
+      <c r="M13">
+        <v>2.85722770690918</v>
+      </c>
+      <c r="N13">
+        <v>0.5249999999999999</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>0.8</v>
+      </c>
+      <c r="Q13">
         <v>0.9</v>
       </c>
-      <c r="K13">
-        <v>0.1</v>
-      </c>
-      <c r="L13">
-        <v>1.0125</v>
-      </c>
-      <c r="M13">
-        <v>0.1</v>
-      </c>
-      <c r="N13">
-        <v>0.1</v>
-      </c>
-      <c r="O13">
-        <v>1</v>
-      </c>
-      <c r="P13">
-        <v>0.1</v>
-      </c>
-      <c r="Q13">
-        <v>0.1</v>
-      </c>
       <c r="R13">
-        <v>1.7125</v>
+        <v>1</v>
       </c>
       <c r="S13">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="T13">
-        <v>0.1</v>
+        <v>0.9</v>
       </c>
       <c r="U13">
-        <v>1.475</v>
+        <v>1</v>
       </c>
       <c r="V13">
         <v>0.1</v>
       </c>
       <c r="W13">
+        <v>0.575</v>
+      </c>
+      <c r="X13">
+        <v>1</v>
+      </c>
+      <c r="Y13">
         <v>0.1</v>
       </c>
-      <c r="X13">
-        <v>0.75</v>
-      </c>
-      <c r="Y13">
-        <v>0.75</v>
-      </c>
       <c r="Z13">
-        <v>0.1</v>
+        <v>0.2374999999999999</v>
       </c>
       <c r="AA13">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:27">
@@ -1978,76 +1990,76 @@
         <v>1</v>
       </c>
       <c r="D14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="E14">
         <v>1</v>
       </c>
       <c r="F14">
-        <v>1.8125</v>
+        <v>1</v>
       </c>
       <c r="G14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>1.475</v>
+        <v>1</v>
       </c>
       <c r="I14">
-        <v>4.193884277343749</v>
+        <v>1</v>
       </c>
       <c r="J14">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="K14">
         <v>1</v>
       </c>
       <c r="L14">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="M14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="N14">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="O14">
-        <v>0.60625</v>
+        <v>1</v>
       </c>
       <c r="P14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="Q14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="R14">
-        <v>2.57724609375</v>
+        <v>1</v>
       </c>
       <c r="S14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="T14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="U14">
-        <v>4.535011291503906</v>
+        <v>1</v>
       </c>
       <c r="V14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="W14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="X14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="Y14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="Z14">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="AA14">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:27">
@@ -3274,76 +3286,76 @@
         <v>1</v>
       </c>
       <c r="D30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="G30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="H30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="I30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="J30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="K30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="L30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="M30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="N30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="O30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="P30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="Q30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="R30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="S30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="T30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="U30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="V30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="W30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="X30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="Y30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="Z30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="AA30">
-        <v>1</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="31" spans="1:27">
@@ -4732,76 +4744,76 @@
         <v>1</v>
       </c>
       <c r="D48">
-        <v>1</v>
+        <v>0.07784846305847154</v>
       </c>
       <c r="E48">
-        <v>1</v>
+        <v>2.347647125990987</v>
       </c>
       <c r="F48">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G48">
-        <v>1</v>
+        <v>0.03569866733551025</v>
       </c>
       <c r="H48">
-        <v>1</v>
+        <v>0.94388671875</v>
       </c>
       <c r="I48">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="J48">
-        <v>1</v>
+        <v>1.49325927734375</v>
       </c>
       <c r="K48">
-        <v>1</v>
+        <v>6.784080180466175</v>
       </c>
       <c r="L48">
-        <v>1</v>
+        <v>1.797608623504639</v>
       </c>
       <c r="M48">
-        <v>1</v>
+        <v>0.8387500000000001</v>
       </c>
       <c r="N48">
-        <v>1</v>
+        <v>4.190825419127941</v>
       </c>
       <c r="O48">
-        <v>1</v>
+        <v>1.804707641601563</v>
       </c>
       <c r="P48">
-        <v>1</v>
+        <v>1.191767578125</v>
       </c>
       <c r="Q48">
-        <v>1</v>
+        <v>7.376191635131836</v>
       </c>
       <c r="R48">
-        <v>1</v>
+        <v>1.568143908441438</v>
       </c>
       <c r="S48">
-        <v>1</v>
+        <v>0.76796875</v>
       </c>
       <c r="T48">
-        <v>1</v>
+        <v>4.475347220897674</v>
       </c>
       <c r="U48">
-        <v>1</v>
+        <v>1.725154495239258</v>
       </c>
       <c r="V48">
-        <v>1</v>
+        <v>1.6812744140625</v>
       </c>
       <c r="W48">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="X48">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Y48">
-        <v>1</v>
+        <v>0.9975000000000001</v>
       </c>
       <c r="Z48">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="AA48">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:27">
@@ -6532,28 +6544,28 @@
         <v>1</v>
       </c>
       <c r="J70">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="K70">
         <v>1</v>
       </c>
       <c r="L70">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="M70">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="N70">
         <v>1</v>
       </c>
       <c r="O70">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="P70">
         <v>1</v>
       </c>
       <c r="Q70">
-        <v>1</v>
+        <v>0.9500000000000001</v>
       </c>
       <c r="R70">
         <v>1</v>
@@ -6562,7 +6574,7 @@
         <v>1</v>
       </c>
       <c r="T70">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="U70">
         <v>1</v>
@@ -6571,16 +6583,16 @@
         <v>1</v>
       </c>
       <c r="W70">
-        <v>1</v>
+        <v>0.825</v>
       </c>
       <c r="X70">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="Y70">
         <v>1</v>
       </c>
       <c r="Z70">
-        <v>1</v>
+        <v>1.15625</v>
       </c>
       <c r="AA70">
         <v>1</v>
@@ -13151,73 +13163,329 @@
       <c r="A152" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="B152" s="1" t="s">
-        <v>5</v>
-      </c>
+      <c r="B152" s="1"/>
       <c r="C152">
         <v>1</v>
       </c>
       <c r="D152">
         <v>1</v>
       </c>
+      <c r="E152">
+        <v>1</v>
+      </c>
+      <c r="F152">
+        <v>1</v>
+      </c>
       <c r="G152">
+        <v>1</v>
+      </c>
+      <c r="H152">
+        <v>1</v>
+      </c>
+      <c r="I152">
+        <v>1</v>
+      </c>
+      <c r="J152">
+        <v>1</v>
+      </c>
+      <c r="K152">
+        <v>1</v>
+      </c>
+      <c r="L152">
+        <v>1</v>
+      </c>
+      <c r="M152">
+        <v>1</v>
+      </c>
+      <c r="N152">
+        <v>1</v>
+      </c>
+      <c r="O152">
+        <v>1</v>
+      </c>
+      <c r="P152">
+        <v>1</v>
+      </c>
+      <c r="Q152">
+        <v>1</v>
+      </c>
+      <c r="R152">
+        <v>1</v>
+      </c>
+      <c r="S152">
+        <v>1</v>
+      </c>
+      <c r="T152">
+        <v>1</v>
+      </c>
+      <c r="U152">
+        <v>1</v>
+      </c>
+      <c r="V152">
+        <v>1</v>
+      </c>
+      <c r="W152">
+        <v>1</v>
+      </c>
+      <c r="X152">
+        <v>1</v>
+      </c>
+      <c r="Y152">
+        <v>1</v>
+      </c>
+      <c r="Z152">
+        <v>1</v>
+      </c>
+      <c r="AA152">
         <v>1</v>
       </c>
     </row>
     <row r="153" spans="1:27">
       <c r="A153" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B153" s="1" t="s">
-        <v>11</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="B153" s="1"/>
       <c r="C153">
         <v>1</v>
       </c>
+      <c r="D153">
+        <v>1</v>
+      </c>
+      <c r="E153">
+        <v>1</v>
+      </c>
+      <c r="F153">
+        <v>1</v>
+      </c>
+      <c r="G153">
+        <v>1</v>
+      </c>
+      <c r="H153">
+        <v>1</v>
+      </c>
+      <c r="I153">
+        <v>1</v>
+      </c>
       <c r="J153">
         <v>1</v>
       </c>
+      <c r="K153">
+        <v>1</v>
+      </c>
+      <c r="L153">
+        <v>1</v>
+      </c>
       <c r="M153">
+        <v>1</v>
+      </c>
+      <c r="N153">
+        <v>1</v>
+      </c>
+      <c r="O153">
+        <v>1</v>
+      </c>
+      <c r="P153">
+        <v>1</v>
+      </c>
+      <c r="Q153">
+        <v>1</v>
+      </c>
+      <c r="R153">
+        <v>1</v>
+      </c>
+      <c r="S153">
+        <v>1</v>
+      </c>
+      <c r="T153">
+        <v>1</v>
+      </c>
+      <c r="U153">
+        <v>1</v>
+      </c>
+      <c r="V153">
+        <v>1</v>
+      </c>
+      <c r="W153">
+        <v>1</v>
+      </c>
+      <c r="X153">
+        <v>1</v>
+      </c>
+      <c r="Y153">
+        <v>1</v>
+      </c>
+      <c r="Z153">
+        <v>1</v>
+      </c>
+      <c r="AA153">
         <v>1</v>
       </c>
     </row>
     <row r="154" spans="1:27">
       <c r="A154" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B154" s="1" t="s">
-        <v>17</v>
-      </c>
+        <v>179</v>
+      </c>
+      <c r="B154" s="1"/>
       <c r="C154">
         <v>1</v>
       </c>
+      <c r="D154">
+        <v>1</v>
+      </c>
+      <c r="E154">
+        <v>1</v>
+      </c>
+      <c r="F154">
+        <v>1</v>
+      </c>
+      <c r="G154">
+        <v>1</v>
+      </c>
+      <c r="H154">
+        <v>1</v>
+      </c>
+      <c r="I154">
+        <v>1</v>
+      </c>
+      <c r="J154">
+        <v>1</v>
+      </c>
+      <c r="K154">
+        <v>1</v>
+      </c>
+      <c r="L154">
+        <v>1</v>
+      </c>
+      <c r="M154">
+        <v>1</v>
+      </c>
+      <c r="N154">
+        <v>1</v>
+      </c>
+      <c r="O154">
+        <v>1</v>
+      </c>
       <c r="P154">
         <v>1</v>
       </c>
+      <c r="Q154">
+        <v>1</v>
+      </c>
+      <c r="R154">
+        <v>1</v>
+      </c>
       <c r="S154">
+        <v>1</v>
+      </c>
+      <c r="T154">
+        <v>1</v>
+      </c>
+      <c r="U154">
+        <v>1</v>
+      </c>
+      <c r="V154">
+        <v>1</v>
+      </c>
+      <c r="W154">
+        <v>1</v>
+      </c>
+      <c r="X154">
+        <v>1</v>
+      </c>
+      <c r="Y154">
+        <v>1</v>
+      </c>
+      <c r="Z154">
+        <v>1</v>
+      </c>
+      <c r="AA154">
         <v>1</v>
       </c>
     </row>
     <row r="155" spans="1:27">
       <c r="A155" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B155" s="1" t="s">
-        <v>23</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="B155" s="1"/>
       <c r="C155">
         <v>1</v>
       </c>
+      <c r="D155">
+        <v>1</v>
+      </c>
+      <c r="E155">
+        <v>1</v>
+      </c>
+      <c r="F155">
+        <v>1</v>
+      </c>
+      <c r="G155">
+        <v>1</v>
+      </c>
+      <c r="H155">
+        <v>1</v>
+      </c>
+      <c r="I155">
+        <v>1</v>
+      </c>
+      <c r="J155">
+        <v>1</v>
+      </c>
+      <c r="K155">
+        <v>1</v>
+      </c>
+      <c r="L155">
+        <v>1</v>
+      </c>
+      <c r="M155">
+        <v>1</v>
+      </c>
+      <c r="N155">
+        <v>1</v>
+      </c>
+      <c r="O155">
+        <v>1</v>
+      </c>
+      <c r="P155">
+        <v>1</v>
+      </c>
+      <c r="Q155">
+        <v>1</v>
+      </c>
+      <c r="R155">
+        <v>1</v>
+      </c>
+      <c r="S155">
+        <v>1</v>
+      </c>
+      <c r="T155">
+        <v>1</v>
+      </c>
+      <c r="U155">
+        <v>1</v>
+      </c>
       <c r="V155">
         <v>1</v>
       </c>
+      <c r="W155">
+        <v>1</v>
+      </c>
+      <c r="X155">
+        <v>1</v>
+      </c>
       <c r="Y155">
+        <v>1</v>
+      </c>
+      <c r="Z155">
+        <v>1</v>
+      </c>
+      <c r="AA155">
         <v>1</v>
       </c>
     </row>
     <row r="156" spans="1:27">
       <c r="A156" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B156" s="1" t="s">
         <v>1</v>
@@ -13226,30 +13494,15 @@
         <v>1</v>
       </c>
       <c r="D156">
-        <v>1</v>
-      </c>
-      <c r="E156">
-        <v>1</v>
-      </c>
-      <c r="F156">
-        <v>1</v>
-      </c>
-      <c r="G156">
-        <v>1</v>
-      </c>
-      <c r="H156">
-        <v>1</v>
-      </c>
-      <c r="I156">
         <v>1</v>
       </c>
     </row>
     <row r="157" spans="1:27">
       <c r="A157" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C157">
         <v>1</v>
@@ -13257,637 +13510,589 @@
       <c r="D157">
         <v>1</v>
       </c>
-      <c r="E157">
-        <v>1</v>
-      </c>
-      <c r="F157">
-        <v>1</v>
-      </c>
       <c r="G157">
-        <v>1</v>
-      </c>
-      <c r="H157">
-        <v>1</v>
-      </c>
-      <c r="I157">
         <v>1</v>
       </c>
     </row>
     <row r="158" spans="1:27">
       <c r="A158" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C158">
         <v>1</v>
       </c>
-      <c r="D158">
-        <v>1</v>
-      </c>
-      <c r="E158">
-        <v>1</v>
-      </c>
-      <c r="F158">
-        <v>1</v>
-      </c>
-      <c r="G158">
-        <v>1</v>
-      </c>
-      <c r="H158">
-        <v>1</v>
-      </c>
-      <c r="I158">
+      <c r="J158">
+        <v>1</v>
+      </c>
+      <c r="M158">
         <v>1</v>
       </c>
     </row>
     <row r="159" spans="1:27">
       <c r="A159" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C159">
         <v>1</v>
       </c>
-      <c r="D159">
-        <v>1</v>
-      </c>
-      <c r="E159">
-        <v>1</v>
-      </c>
-      <c r="F159">
-        <v>1</v>
-      </c>
-      <c r="G159">
-        <v>1</v>
-      </c>
-      <c r="H159">
-        <v>1</v>
-      </c>
-      <c r="I159">
+      <c r="J159">
+        <v>1</v>
+      </c>
+      <c r="M159">
         <v>1</v>
       </c>
     </row>
     <row r="160" spans="1:27">
       <c r="A160" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B160" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C160">
+        <v>1</v>
+      </c>
+      <c r="J160">
+        <v>1</v>
+      </c>
+      <c r="M160">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161" spans="1:21">
+      <c r="A161" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C161">
+        <v>1</v>
+      </c>
+      <c r="D161">
+        <v>1</v>
+      </c>
+      <c r="E161">
+        <v>1</v>
+      </c>
+      <c r="F161">
+        <v>1</v>
+      </c>
+      <c r="G161">
+        <v>1</v>
+      </c>
+      <c r="H161">
+        <v>1</v>
+      </c>
+      <c r="I161">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162" spans="1:21">
+      <c r="A162" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C162">
+        <v>1</v>
+      </c>
+      <c r="D162">
+        <v>1</v>
+      </c>
+      <c r="E162">
+        <v>1</v>
+      </c>
+      <c r="F162">
+        <v>1</v>
+      </c>
+      <c r="G162">
+        <v>1</v>
+      </c>
+      <c r="H162">
+        <v>1</v>
+      </c>
+      <c r="I162">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:21">
+      <c r="A163" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C163">
+        <v>1</v>
+      </c>
+      <c r="D163">
+        <v>1</v>
+      </c>
+      <c r="E163">
+        <v>1</v>
+      </c>
+      <c r="F163">
+        <v>1</v>
+      </c>
+      <c r="G163">
+        <v>1</v>
+      </c>
+      <c r="H163">
+        <v>1</v>
+      </c>
+      <c r="I163">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164" spans="1:21">
+      <c r="A164" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B164" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C164">
+        <v>1</v>
+      </c>
+      <c r="D164">
+        <v>1</v>
+      </c>
+      <c r="E164">
+        <v>1</v>
+      </c>
+      <c r="F164">
+        <v>1</v>
+      </c>
+      <c r="G164">
+        <v>1</v>
+      </c>
+      <c r="H164">
+        <v>1</v>
+      </c>
+      <c r="I164">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:21">
+      <c r="A165" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B165" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C160">
-        <v>1</v>
-      </c>
-      <c r="D160">
-        <v>1</v>
-      </c>
-      <c r="E160">
-        <v>1</v>
-      </c>
-      <c r="F160">
-        <v>1</v>
-      </c>
-      <c r="G160">
-        <v>1</v>
-      </c>
-      <c r="H160">
-        <v>1</v>
-      </c>
-      <c r="I160">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="161" spans="1:27">
-      <c r="A161" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B161" s="1" t="s">
+      <c r="C165">
+        <v>1</v>
+      </c>
+      <c r="D165">
+        <v>1</v>
+      </c>
+      <c r="E165">
+        <v>1</v>
+      </c>
+      <c r="F165">
+        <v>1</v>
+      </c>
+      <c r="G165">
+        <v>1</v>
+      </c>
+      <c r="H165">
+        <v>1</v>
+      </c>
+      <c r="I165">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166" spans="1:21">
+      <c r="A166" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B166" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C161">
-        <v>1</v>
-      </c>
-      <c r="D161">
-        <v>1</v>
-      </c>
-      <c r="E161">
-        <v>1</v>
-      </c>
-      <c r="F161">
-        <v>1</v>
-      </c>
-      <c r="G161">
-        <v>1</v>
-      </c>
-      <c r="H161">
-        <v>1</v>
-      </c>
-      <c r="I161">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="162" spans="1:27">
-      <c r="A162" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B162" s="1" t="s">
+      <c r="C166">
+        <v>1</v>
+      </c>
+      <c r="D166">
+        <v>1</v>
+      </c>
+      <c r="E166">
+        <v>1</v>
+      </c>
+      <c r="F166">
+        <v>1</v>
+      </c>
+      <c r="G166">
+        <v>1</v>
+      </c>
+      <c r="H166">
+        <v>1</v>
+      </c>
+      <c r="I166">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:21">
+      <c r="A167" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B167" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C162">
-        <v>1</v>
-      </c>
-      <c r="J162">
-        <v>1</v>
-      </c>
-      <c r="K162">
-        <v>1</v>
-      </c>
-      <c r="L162">
-        <v>1</v>
-      </c>
-      <c r="M162">
-        <v>1</v>
-      </c>
-      <c r="N162">
-        <v>1</v>
-      </c>
-      <c r="O162">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="163" spans="1:27">
-      <c r="A163" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B163" s="1" t="s">
+      <c r="C167">
+        <v>1</v>
+      </c>
+      <c r="J167">
+        <v>1</v>
+      </c>
+      <c r="K167">
+        <v>1</v>
+      </c>
+      <c r="L167">
+        <v>1</v>
+      </c>
+      <c r="M167">
+        <v>1</v>
+      </c>
+      <c r="N167">
+        <v>1</v>
+      </c>
+      <c r="O167">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168" spans="1:21">
+      <c r="A168" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B168" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C163">
-        <v>1</v>
-      </c>
-      <c r="J163">
-        <v>1</v>
-      </c>
-      <c r="K163">
-        <v>1</v>
-      </c>
-      <c r="L163">
-        <v>1</v>
-      </c>
-      <c r="M163">
-        <v>1</v>
-      </c>
-      <c r="N163">
-        <v>1</v>
-      </c>
-      <c r="O163">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="164" spans="1:27">
-      <c r="A164" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B164" s="1" t="s">
+      <c r="C168">
+        <v>1</v>
+      </c>
+      <c r="J168">
+        <v>1</v>
+      </c>
+      <c r="K168">
+        <v>1</v>
+      </c>
+      <c r="L168">
+        <v>1</v>
+      </c>
+      <c r="M168">
+        <v>1</v>
+      </c>
+      <c r="N168">
+        <v>1</v>
+      </c>
+      <c r="O168">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169" spans="1:21">
+      <c r="A169" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B169" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C164">
-        <v>1</v>
-      </c>
-      <c r="J164">
-        <v>1</v>
-      </c>
-      <c r="K164">
-        <v>1</v>
-      </c>
-      <c r="L164">
-        <v>1</v>
-      </c>
-      <c r="M164">
-        <v>1</v>
-      </c>
-      <c r="N164">
-        <v>1</v>
-      </c>
-      <c r="O164">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="165" spans="1:27">
-      <c r="A165" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B165" s="1" t="s">
+      <c r="C169">
+        <v>1</v>
+      </c>
+      <c r="J169">
+        <v>1</v>
+      </c>
+      <c r="K169">
+        <v>1</v>
+      </c>
+      <c r="L169">
+        <v>1</v>
+      </c>
+      <c r="M169">
+        <v>1</v>
+      </c>
+      <c r="N169">
+        <v>1</v>
+      </c>
+      <c r="O169">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170" spans="1:21">
+      <c r="A170" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B170" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C165">
-        <v>1</v>
-      </c>
-      <c r="J165">
-        <v>1</v>
-      </c>
-      <c r="K165">
-        <v>1</v>
-      </c>
-      <c r="L165">
-        <v>1</v>
-      </c>
-      <c r="M165">
-        <v>1</v>
-      </c>
-      <c r="N165">
-        <v>1</v>
-      </c>
-      <c r="O165">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="166" spans="1:27">
-      <c r="A166" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B166" s="1" t="s">
+      <c r="C170">
+        <v>1</v>
+      </c>
+      <c r="J170">
+        <v>1</v>
+      </c>
+      <c r="K170">
+        <v>1</v>
+      </c>
+      <c r="L170">
+        <v>1</v>
+      </c>
+      <c r="M170">
+        <v>1</v>
+      </c>
+      <c r="N170">
+        <v>1</v>
+      </c>
+      <c r="O170">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" spans="1:21">
+      <c r="A171" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B171" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C166">
-        <v>1</v>
-      </c>
-      <c r="J166">
-        <v>1</v>
-      </c>
-      <c r="K166">
-        <v>1</v>
-      </c>
-      <c r="L166">
-        <v>1</v>
-      </c>
-      <c r="M166">
-        <v>1</v>
-      </c>
-      <c r="N166">
-        <v>1</v>
-      </c>
-      <c r="O166">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="167" spans="1:27">
-      <c r="A167" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B167" s="1" t="s">
+      <c r="C171">
+        <v>1</v>
+      </c>
+      <c r="J171">
+        <v>1</v>
+      </c>
+      <c r="K171">
+        <v>1</v>
+      </c>
+      <c r="L171">
+        <v>1</v>
+      </c>
+      <c r="M171">
+        <v>1</v>
+      </c>
+      <c r="N171">
+        <v>1</v>
+      </c>
+      <c r="O171">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" spans="1:21">
+      <c r="A172" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B172" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C167">
-        <v>1</v>
-      </c>
-      <c r="J167">
-        <v>1</v>
-      </c>
-      <c r="K167">
-        <v>1</v>
-      </c>
-      <c r="L167">
-        <v>1</v>
-      </c>
-      <c r="M167">
-        <v>1</v>
-      </c>
-      <c r="N167">
-        <v>1</v>
-      </c>
-      <c r="O167">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="168" spans="1:27">
-      <c r="A168" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B168" s="1" t="s">
+      <c r="C172">
+        <v>1</v>
+      </c>
+      <c r="J172">
+        <v>1</v>
+      </c>
+      <c r="K172">
+        <v>1</v>
+      </c>
+      <c r="L172">
+        <v>1</v>
+      </c>
+      <c r="M172">
+        <v>1</v>
+      </c>
+      <c r="N172">
+        <v>1</v>
+      </c>
+      <c r="O172">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173" spans="1:21">
+      <c r="A173" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B173" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C168">
-        <v>1</v>
-      </c>
-      <c r="P168">
-        <v>1</v>
-      </c>
-      <c r="Q168">
-        <v>1</v>
-      </c>
-      <c r="R168">
-        <v>1</v>
-      </c>
-      <c r="S168">
-        <v>1</v>
-      </c>
-      <c r="T168">
-        <v>1</v>
-      </c>
-      <c r="U168">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="169" spans="1:27">
-      <c r="A169" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B169" s="1" t="s">
+      <c r="C173">
+        <v>1</v>
+      </c>
+      <c r="P173">
+        <v>1</v>
+      </c>
+      <c r="Q173">
+        <v>1</v>
+      </c>
+      <c r="R173">
+        <v>1</v>
+      </c>
+      <c r="S173">
+        <v>1</v>
+      </c>
+      <c r="T173">
+        <v>1</v>
+      </c>
+      <c r="U173">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:21">
+      <c r="A174" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B174" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C169">
-        <v>1</v>
-      </c>
-      <c r="P169">
-        <v>1</v>
-      </c>
-      <c r="Q169">
-        <v>1</v>
-      </c>
-      <c r="R169">
-        <v>1</v>
-      </c>
-      <c r="S169">
-        <v>1</v>
-      </c>
-      <c r="T169">
-        <v>1</v>
-      </c>
-      <c r="U169">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="170" spans="1:27">
-      <c r="A170" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B170" s="1" t="s">
+      <c r="C174">
+        <v>1</v>
+      </c>
+      <c r="P174">
+        <v>1</v>
+      </c>
+      <c r="Q174">
+        <v>1</v>
+      </c>
+      <c r="R174">
+        <v>1</v>
+      </c>
+      <c r="S174">
+        <v>1</v>
+      </c>
+      <c r="T174">
+        <v>1</v>
+      </c>
+      <c r="U174">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175" spans="1:21">
+      <c r="A175" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B175" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C170">
-        <v>1</v>
-      </c>
-      <c r="P170">
-        <v>1</v>
-      </c>
-      <c r="Q170">
-        <v>1</v>
-      </c>
-      <c r="R170">
-        <v>1</v>
-      </c>
-      <c r="S170">
-        <v>1</v>
-      </c>
-      <c r="T170">
-        <v>1</v>
-      </c>
-      <c r="U170">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="171" spans="1:27">
-      <c r="A171" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B171" s="1" t="s">
+      <c r="C175">
+        <v>1</v>
+      </c>
+      <c r="P175">
+        <v>1</v>
+      </c>
+      <c r="Q175">
+        <v>1</v>
+      </c>
+      <c r="R175">
+        <v>1</v>
+      </c>
+      <c r="S175">
+        <v>1</v>
+      </c>
+      <c r="T175">
+        <v>1</v>
+      </c>
+      <c r="U175">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:21">
+      <c r="A176" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B176" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C171">
-        <v>1</v>
-      </c>
-      <c r="P171">
-        <v>1</v>
-      </c>
-      <c r="Q171">
-        <v>1</v>
-      </c>
-      <c r="R171">
-        <v>1</v>
-      </c>
-      <c r="S171">
-        <v>1</v>
-      </c>
-      <c r="T171">
-        <v>1</v>
-      </c>
-      <c r="U171">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="172" spans="1:27">
-      <c r="A172" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B172" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C172">
-        <v>1</v>
-      </c>
-      <c r="P172">
-        <v>1</v>
-      </c>
-      <c r="Q172">
-        <v>1</v>
-      </c>
-      <c r="R172">
-        <v>1</v>
-      </c>
-      <c r="S172">
-        <v>1</v>
-      </c>
-      <c r="T172">
-        <v>1</v>
-      </c>
-      <c r="U172">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="173" spans="1:27">
-      <c r="A173" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B173" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C173">
-        <v>1</v>
-      </c>
-      <c r="P173">
-        <v>1</v>
-      </c>
-      <c r="Q173">
-        <v>1</v>
-      </c>
-      <c r="R173">
-        <v>1</v>
-      </c>
-      <c r="S173">
-        <v>1</v>
-      </c>
-      <c r="T173">
-        <v>1</v>
-      </c>
-      <c r="U173">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="174" spans="1:27">
-      <c r="A174" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B174" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C174">
-        <v>1</v>
-      </c>
-      <c r="V174">
-        <v>1</v>
-      </c>
-      <c r="W174">
-        <v>1</v>
-      </c>
-      <c r="X174">
-        <v>1</v>
-      </c>
-      <c r="Y174">
-        <v>1</v>
-      </c>
-      <c r="Z174">
-        <v>1</v>
-      </c>
-      <c r="AA174">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="175" spans="1:27">
-      <c r="A175" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B175" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C175">
-        <v>1</v>
-      </c>
-      <c r="V175">
-        <v>1</v>
-      </c>
-      <c r="W175">
-        <v>1</v>
-      </c>
-      <c r="X175">
-        <v>1</v>
-      </c>
-      <c r="Y175">
-        <v>1</v>
-      </c>
-      <c r="Z175">
-        <v>1</v>
-      </c>
-      <c r="AA175">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="176" spans="1:27">
-      <c r="A176" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B176" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="C176">
         <v>1</v>
       </c>
-      <c r="V176">
-        <v>1</v>
-      </c>
-      <c r="W176">
-        <v>1</v>
-      </c>
-      <c r="X176">
-        <v>1</v>
-      </c>
-      <c r="Y176">
-        <v>1</v>
-      </c>
-      <c r="Z176">
-        <v>1</v>
-      </c>
-      <c r="AA176">
+      <c r="P176">
+        <v>1</v>
+      </c>
+      <c r="Q176">
+        <v>1</v>
+      </c>
+      <c r="R176">
+        <v>1</v>
+      </c>
+      <c r="S176">
+        <v>1</v>
+      </c>
+      <c r="T176">
+        <v>1</v>
+      </c>
+      <c r="U176">
         <v>1</v>
       </c>
     </row>
     <row r="177" spans="1:27">
       <c r="A177" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C177">
         <v>1</v>
       </c>
-      <c r="V177">
-        <v>1</v>
-      </c>
-      <c r="W177">
-        <v>1</v>
-      </c>
-      <c r="X177">
-        <v>1</v>
-      </c>
-      <c r="Y177">
-        <v>1</v>
-      </c>
-      <c r="Z177">
-        <v>1</v>
-      </c>
-      <c r="AA177">
+      <c r="P177">
+        <v>1</v>
+      </c>
+      <c r="Q177">
+        <v>1</v>
+      </c>
+      <c r="R177">
+        <v>1</v>
+      </c>
+      <c r="S177">
+        <v>1</v>
+      </c>
+      <c r="T177">
+        <v>1</v>
+      </c>
+      <c r="U177">
         <v>1</v>
       </c>
     </row>
     <row r="178" spans="1:27">
       <c r="A178" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C178">
         <v>1</v>
       </c>
-      <c r="V178">
-        <v>1</v>
-      </c>
-      <c r="W178">
-        <v>1</v>
-      </c>
-      <c r="X178">
-        <v>1</v>
-      </c>
-      <c r="Y178">
-        <v>1</v>
-      </c>
-      <c r="Z178">
-        <v>1</v>
-      </c>
-      <c r="AA178">
+      <c r="P178">
+        <v>1</v>
+      </c>
+      <c r="Q178">
+        <v>1</v>
+      </c>
+      <c r="R178">
+        <v>1</v>
+      </c>
+      <c r="S178">
+        <v>1</v>
+      </c>
+      <c r="T178">
+        <v>1</v>
+      </c>
+      <c r="U178">
         <v>1</v>
       </c>
     </row>
     <row r="179" spans="1:27">
       <c r="A179" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C179">
         <v>1</v>
@@ -13913,225 +14118,370 @@
     </row>
     <row r="180" spans="1:27">
       <c r="A180" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C180">
         <v>1</v>
       </c>
-      <c r="E180">
+      <c r="V180">
+        <v>1</v>
+      </c>
+      <c r="W180">
+        <v>1</v>
+      </c>
+      <c r="X180">
+        <v>1</v>
+      </c>
+      <c r="Y180">
+        <v>1</v>
+      </c>
+      <c r="Z180">
+        <v>1</v>
+      </c>
+      <c r="AA180">
         <v>1</v>
       </c>
     </row>
     <row r="181" spans="1:27">
       <c r="A181" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="C181">
         <v>1</v>
       </c>
-      <c r="F181">
+      <c r="V181">
+        <v>1</v>
+      </c>
+      <c r="W181">
+        <v>1</v>
+      </c>
+      <c r="X181">
+        <v>1</v>
+      </c>
+      <c r="Y181">
+        <v>1</v>
+      </c>
+      <c r="Z181">
+        <v>1</v>
+      </c>
+      <c r="AA181">
         <v>1</v>
       </c>
     </row>
     <row r="182" spans="1:27">
       <c r="A182" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C182">
         <v>1</v>
       </c>
-      <c r="H182">
+      <c r="V182">
+        <v>1</v>
+      </c>
+      <c r="W182">
+        <v>1</v>
+      </c>
+      <c r="X182">
+        <v>1</v>
+      </c>
+      <c r="Y182">
+        <v>1</v>
+      </c>
+      <c r="Z182">
+        <v>1</v>
+      </c>
+      <c r="AA182">
         <v>1</v>
       </c>
     </row>
     <row r="183" spans="1:27">
       <c r="A183" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="C183">
         <v>1</v>
       </c>
-      <c r="I183">
+      <c r="V183">
+        <v>1</v>
+      </c>
+      <c r="W183">
+        <v>1</v>
+      </c>
+      <c r="X183">
+        <v>1</v>
+      </c>
+      <c r="Y183">
+        <v>1</v>
+      </c>
+      <c r="Z183">
+        <v>1</v>
+      </c>
+      <c r="AA183">
         <v>1</v>
       </c>
     </row>
     <row r="184" spans="1:27">
       <c r="A184" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="C184">
         <v>1</v>
       </c>
-      <c r="K184">
+      <c r="V184">
+        <v>1</v>
+      </c>
+      <c r="W184">
+        <v>1</v>
+      </c>
+      <c r="X184">
+        <v>1</v>
+      </c>
+      <c r="Y184">
+        <v>1</v>
+      </c>
+      <c r="Z184">
+        <v>1</v>
+      </c>
+      <c r="AA184">
         <v>1</v>
       </c>
     </row>
     <row r="185" spans="1:27">
       <c r="A185" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C185">
         <v>1</v>
       </c>
-      <c r="L185">
+      <c r="E185">
         <v>1</v>
       </c>
     </row>
     <row r="186" spans="1:27">
       <c r="A186" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C186">
         <v>1</v>
       </c>
-      <c r="N186">
+      <c r="F186">
         <v>1</v>
       </c>
     </row>
     <row r="187" spans="1:27">
       <c r="A187" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C187">
         <v>1</v>
       </c>
-      <c r="O187">
+      <c r="H187">
         <v>1</v>
       </c>
     </row>
     <row r="188" spans="1:27">
       <c r="A188" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C188">
         <v>1</v>
       </c>
-      <c r="Q188">
+      <c r="I188">
         <v>1</v>
       </c>
     </row>
     <row r="189" spans="1:27">
       <c r="A189" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C189">
         <v>1</v>
       </c>
-      <c r="R189">
+      <c r="K189">
         <v>1</v>
       </c>
     </row>
     <row r="190" spans="1:27">
       <c r="A190" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C190">
         <v>1</v>
       </c>
-      <c r="T190">
+      <c r="L190">
         <v>1</v>
       </c>
     </row>
     <row r="191" spans="1:27">
       <c r="A191" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C191">
         <v>1</v>
       </c>
-      <c r="U191">
+      <c r="N191">
         <v>1</v>
       </c>
     </row>
     <row r="192" spans="1:27">
       <c r="A192" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C192">
         <v>1</v>
       </c>
-      <c r="W192">
+      <c r="O192">
         <v>1</v>
       </c>
     </row>
     <row r="193" spans="1:27">
       <c r="A193" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C193">
         <v>1</v>
       </c>
-      <c r="X193">
+      <c r="Q193">
         <v>1</v>
       </c>
     </row>
     <row r="194" spans="1:27">
       <c r="A194" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C194">
         <v>1</v>
       </c>
-      <c r="Z194">
+      <c r="R194">
         <v>1</v>
       </c>
     </row>
     <row r="195" spans="1:27">
       <c r="A195" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B195" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C195">
+        <v>1</v>
+      </c>
+      <c r="T195">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196" spans="1:27">
+      <c r="A196" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B196" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C196">
+        <v>1</v>
+      </c>
+      <c r="U196">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197" spans="1:27">
+      <c r="A197" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B197" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C197">
+        <v>1</v>
+      </c>
+      <c r="W197">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198" spans="1:27">
+      <c r="A198" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B198" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C198">
+        <v>1</v>
+      </c>
+      <c r="X198">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:27">
+      <c r="A199" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B199" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C199">
+        <v>1</v>
+      </c>
+      <c r="Z199">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:27">
+      <c r="A200" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B200" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C195">
-        <v>1</v>
-      </c>
-      <c r="AA195">
+      <c r="C200">
+        <v>1</v>
+      </c>
+      <c r="AA200">
         <v>1</v>
       </c>
     </row>

</xml_diff>